<commit_message>
#3 Pull Up Resistor added in led Switch and Fresh Deliverables Generated Also.e Ge
</commit_message>
<xml_diff>
--- a/Design Files/Main-Board-v1.0/BOM/Client-BOM-Main Board - v1.0.xlsx
+++ b/Design Files/Main-Board-v1.0/BOM/Client-BOM-Main Board - v1.0.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="125">
   <si>
     <t>#</t>
   </si>
@@ -117,7 +117,7 @@
     <t>R3</t>
   </si>
   <si>
-    <t>R4, R5, R6, R8, R9, R10</t>
+    <t>R4, R5, R6, R8, R9, R10, R12</t>
   </si>
   <si>
     <t>R7, R11</t>
@@ -394,9 +394,6 @@
   </si>
   <si>
     <t>Custom</t>
-  </si>
-  <si>
-    <t>USB Connector</t>
   </si>
 </sst>
 </file>
@@ -894,10 +891,10 @@
   <cols>
     <col min="2" max="2" width="3.140625" style="4" customWidth="1"/>
     <col min="3" max="3" width="18.7109375" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -1174,14 +1171,14 @@
       </c>
       <c r="K9" s="7"/>
     </row>
-    <row r="10" spans="1:11" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="11">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>125</v>
+        <v>6</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>25</v>
@@ -1221,7 +1218,7 @@
       <c r="E11" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="F11" s="9" t="s">
         <v>124</v>
       </c>
       <c r="G11" s="8" t="s">
@@ -1253,7 +1250,7 @@
       <c r="E12" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="F12" s="9" t="s">
         <v>124</v>
       </c>
       <c r="G12" s="10" t="s">
@@ -1285,7 +1282,7 @@
       <c r="E13" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="F13" s="9" t="s">
         <v>124</v>
       </c>
       <c r="G13" s="8" t="s">
@@ -1426,7 +1423,7 @@
         <v>117</v>
       </c>
       <c r="J17" s="7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K17" s="7"/>
     </row>
@@ -1477,7 +1474,7 @@
       <c r="E19" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="F19" s="9" t="s">
         <v>124</v>
       </c>
       <c r="G19" s="8" t="s">

</xml_diff>